<commit_message>
feat: Participants Grid with Grouping and Nationality Logic
</commit_message>
<xml_diff>
--- a/inp_Excel/ana_viaggi.xlsx
+++ b/inp_Excel/ana_viaggi.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="210">
   <si>
     <t>VIAGGIO_ID</t>
   </si>
@@ -387,6 +387,15 @@
   </si>
   <si>
     <t>3 GIORNI DI PURO ENDURO</t>
+  </si>
+  <si>
+    <t>PORTOGALLO IN 4X4</t>
+  </si>
+  <si>
+    <t>Un viaggio nel cuore di questa nazione</t>
+  </si>
+  <si>
+    <t>https://www.sardegnafuoritraccia.it/it/tour/fuoristrada-estero/nord-portugal-4x4</t>
   </si>
   <si>
     <t>4X4 - BALCANI ADVENTURE</t>
@@ -760,8 +769,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:W63" totalsRowShown="0" headerRowCount="1">
-  <autoFilter ref="A1:W63"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:W64" totalsRowShown="0" headerRowCount="1">
+  <autoFilter ref="A1:W64"/>
   <tableColumns count="23">
     <tableColumn id="1" name="VIAGGIO_ID"/>
     <tableColumn id="2" name="VIAGGIO_DESCRIZIONE_BREVE"/>
@@ -2817,7 +2826,7 @@
     </row>
     <row r="35" customHeight="1" ht="20">
       <c r="A35" s="5" t="n">
-        <v>23</v>
+        <v>861</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>121</v>
@@ -2826,19 +2835,19 @@
         <v>122</v>
       </c>
       <c r="D35" s="5" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F35" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>1700</v>
+        <v>1500</v>
       </c>
       <c r="H35" s="6" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I35" s="6"/>
       <c r="J35" s="5" t="n">
@@ -2848,16 +2857,16 @@
         <v>14</v>
       </c>
       <c r="L35" s="5" t="n">
-        <v>146</v>
+        <v>177</v>
       </c>
       <c r="M35" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="O35" s="7" t="n">
-        <v>44420.4166319444</v>
+        <v>46031.304849537</v>
       </c>
       <c r="P35" s="6"/>
       <c r="Q35" s="7"/>
@@ -2867,36 +2876,32 @@
       <c r="S35" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T35" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="U35" s="6" t="s">
-        <v>124</v>
-      </c>
+      <c r="T35" s="6"/>
+      <c r="U35" s="6"/>
       <c r="V35" s="6"/>
       <c r="W35" s="6"/>
     </row>
     <row r="36" customHeight="1" ht="20">
       <c r="A36" s="5" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C36" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="D36" s="5" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G36" s="5" t="n">
-        <v>304</v>
+        <v>1700</v>
       </c>
       <c r="H36" s="6" t="s">
         <v>56</v>
@@ -2909,21 +2914,21 @@
         <v>14</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="M36" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O36" s="7" t="n">
-        <v>44420.4193634259</v>
+        <v>44420.4166319444</v>
       </c>
       <c r="P36" s="6"/>
       <c r="Q36" s="7"/>
       <c r="R36" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="S36" s="6" t="s">
         <v>28</v>
@@ -2932,32 +2937,32 @@
         <v>29</v>
       </c>
       <c r="U36" s="6" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="V36" s="6"/>
       <c r="W36" s="6"/>
     </row>
-    <row r="37" customHeight="1" ht="29">
+    <row r="37" customHeight="1" ht="20">
       <c r="A37" s="5" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B37" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="C37" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>130</v>
-      </c>
       <c r="D37" s="5" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F37" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G37" s="5" t="n">
-        <v>1000</v>
+        <v>304</v>
       </c>
       <c r="H37" s="6" t="s">
         <v>56</v>
@@ -2967,10 +2972,10 @@
         <v>1</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>2</v>
+        <v>76</v>
       </c>
       <c r="M37" s="5" t="n">
         <v>10</v>
@@ -2979,12 +2984,12 @@
         <v>26</v>
       </c>
       <c r="O37" s="7" t="n">
-        <v>44420.5078125</v>
+        <v>44420.4193634259</v>
       </c>
       <c r="P37" s="6"/>
       <c r="Q37" s="7"/>
       <c r="R37" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="S37" s="6" t="s">
         <v>28</v>
@@ -2993,45 +2998,45 @@
         <v>29</v>
       </c>
       <c r="U37" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="V37" s="6"/>
       <c r="W37" s="6"/>
     </row>
-    <row r="38" customHeight="1" ht="20">
+    <row r="38" customHeight="1" ht="29">
       <c r="A38" s="5" t="n">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>133</v>
       </c>
       <c r="D38" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G38" s="5" t="n">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="I38" s="6"/>
       <c r="J38" s="5" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="K38" s="5" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L38" s="5" t="n">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="M38" s="5" t="n">
         <v>10</v>
@@ -3040,47 +3045,53 @@
         <v>26</v>
       </c>
       <c r="O38" s="7" t="n">
-        <v>44468.751412037</v>
+        <v>44420.5078125</v>
       </c>
       <c r="P38" s="6"/>
       <c r="Q38" s="7"/>
-      <c r="R38" s="6"/>
+      <c r="R38" s="6" t="s">
+        <v>134</v>
+      </c>
       <c r="S38" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T38" s="6"/>
-      <c r="U38" s="6"/>
+      <c r="T38" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="U38" s="6" t="s">
+        <v>135</v>
+      </c>
       <c r="V38" s="6"/>
       <c r="W38" s="6"/>
     </row>
-    <row r="39" customHeight="1" ht="43,5">
+    <row r="39" customHeight="1" ht="20">
       <c r="A39" s="5" t="n">
-        <v>81</v>
+        <v>61</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D39" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E39" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="F39" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G39" s="5" t="n">
-        <v>205</v>
+        <v>350</v>
       </c>
       <c r="H39" s="6" t="s">
         <v>25</v>
       </c>
       <c r="I39" s="6"/>
       <c r="J39" s="5" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K39" s="5" t="n">
         <v>13</v>
@@ -3095,34 +3106,28 @@
         <v>26</v>
       </c>
       <c r="O39" s="7" t="n">
-        <v>44594.3402662037</v>
+        <v>44468.751412037</v>
       </c>
       <c r="P39" s="6"/>
       <c r="Q39" s="7"/>
-      <c r="R39" s="6" t="s">
-        <v>136</v>
-      </c>
+      <c r="R39" s="6"/>
       <c r="S39" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T39" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="U39" s="6" t="s">
-        <v>138</v>
-      </c>
+      <c r="T39" s="6"/>
+      <c r="U39" s="6"/>
       <c r="V39" s="6"/>
       <c r="W39" s="6"/>
     </row>
-    <row r="40" customHeight="1" ht="29">
+    <row r="40" customHeight="1" ht="43,5">
       <c r="A40" s="5" t="n">
-        <v>101</v>
+        <v>81</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D40" s="5" t="n">
         <v>2</v>
@@ -3134,7 +3139,7 @@
         <v>24</v>
       </c>
       <c r="G40" s="5" t="n">
-        <v>230</v>
+        <v>205</v>
       </c>
       <c r="H40" s="6" t="s">
         <v>25</v>
@@ -3156,34 +3161,34 @@
         <v>26</v>
       </c>
       <c r="O40" s="7" t="n">
-        <v>44615.8342361111</v>
+        <v>44594.3402662037</v>
       </c>
       <c r="P40" s="6"/>
       <c r="Q40" s="7"/>
       <c r="R40" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="S40" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T40" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="U40" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="S40" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T40" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="U40" s="6" t="s">
-        <v>142</v>
       </c>
       <c r="V40" s="6"/>
       <c r="W40" s="6"/>
     </row>
-    <row r="41" customHeight="1" ht="87">
+    <row r="41" customHeight="1" ht="29">
       <c r="A41" s="5" t="n">
-        <v>181</v>
+        <v>101</v>
       </c>
       <c r="B41" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C41" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="D41" s="5" t="n">
         <v>2</v>
@@ -3195,7 +3200,7 @@
         <v>24</v>
       </c>
       <c r="G41" s="5" t="n">
-        <v>210</v>
+        <v>230</v>
       </c>
       <c r="H41" s="6" t="s">
         <v>25</v>
@@ -3217,34 +3222,34 @@
         <v>26</v>
       </c>
       <c r="O41" s="7" t="n">
-        <v>44810.5888425926</v>
+        <v>44615.8342361111</v>
       </c>
       <c r="P41" s="6"/>
       <c r="Q41" s="7"/>
       <c r="R41" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="S41" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T41" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="U41" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="S41" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T41" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="U41" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="V41" s="6"/>
       <c r="W41" s="6"/>
     </row>
-    <row r="42" customHeight="1" ht="43,5">
+    <row r="42" customHeight="1" ht="87">
       <c r="A42" s="5" t="n">
-        <v>201</v>
+        <v>181</v>
       </c>
       <c r="B42" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="D42" s="5" t="n">
         <v>2</v>
@@ -3256,7 +3261,7 @@
         <v>24</v>
       </c>
       <c r="G42" s="5" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="H42" s="6" t="s">
         <v>25</v>
@@ -3278,56 +3283,56 @@
         <v>26</v>
       </c>
       <c r="O42" s="7" t="n">
-        <v>44834.2956712963</v>
+        <v>44810.5888425926</v>
       </c>
       <c r="P42" s="6"/>
       <c r="Q42" s="7"/>
       <c r="R42" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="S42" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T42" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="U42" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="S42" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T42" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="U42" s="6" t="s">
-        <v>150</v>
       </c>
       <c r="V42" s="6"/>
       <c r="W42" s="6"/>
     </row>
     <row r="43" customHeight="1" ht="43,5">
       <c r="A43" s="5" t="n">
-        <v>741</v>
+        <v>201</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="C43" s="6" t="s">
-        <v>152</v>
-      </c>
       <c r="D43" s="5" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E43" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F43" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G43" s="5" t="n">
-        <v>650</v>
+        <v>240</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I43" s="6"/>
       <c r="J43" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K43" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L43" s="5" t="n">
         <v>110</v>
@@ -3336,27 +3341,31 @@
         <v>10</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="O43" s="7" t="n">
-        <v>45951.6437962963</v>
+        <v>44834.2956712963</v>
       </c>
       <c r="P43" s="6"/>
       <c r="Q43" s="7"/>
       <c r="R43" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="S43" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T43" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="U43" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="S43" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T43" s="6"/>
-      <c r="U43" s="6"/>
       <c r="V43" s="6"/>
       <c r="W43" s="6"/>
     </row>
-    <row r="44" customHeight="1" ht="20">
+    <row r="44" customHeight="1" ht="43,5">
       <c r="A44" s="5" t="n">
-        <v>622</v>
+        <v>741</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>154</v>
@@ -3365,10 +3374,10 @@
         <v>155</v>
       </c>
       <c r="D44" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>24</v>
@@ -3396,7 +3405,7 @@
         <v>60</v>
       </c>
       <c r="O44" s="7" t="n">
-        <v>45700.7497453704</v>
+        <v>45951.6437962963</v>
       </c>
       <c r="P44" s="6"/>
       <c r="Q44" s="7"/>
@@ -3413,7 +3422,7 @@
     </row>
     <row r="45" customHeight="1" ht="20">
       <c r="A45" s="5" t="n">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>157</v>
@@ -3422,16 +3431,16 @@
         <v>158</v>
       </c>
       <c r="D45" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E45" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="E45" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="F45" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G45" s="5" t="n">
-        <v>600</v>
+        <v>650</v>
       </c>
       <c r="H45" s="6" t="s">
         <v>56</v>
@@ -3441,19 +3450,19 @@
         <v>1</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="L45" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M45" s="5" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="N45" s="6" t="s">
         <v>60</v>
       </c>
       <c r="O45" s="7" t="n">
-        <v>45700.7520138889</v>
+        <v>45700.7497453704</v>
       </c>
       <c r="P45" s="6"/>
       <c r="Q45" s="7"/>
@@ -3470,7 +3479,7 @@
     </row>
     <row r="46" customHeight="1" ht="20">
       <c r="A46" s="5" t="n">
-        <v>761</v>
+        <v>624</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>160</v>
@@ -3479,16 +3488,16 @@
         <v>161</v>
       </c>
       <c r="D46" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G46" s="5" t="n">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="H46" s="6" t="s">
         <v>56</v>
@@ -3498,23 +3507,25 @@
         <v>1</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="L46" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M46" s="5" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N46" s="6" t="s">
         <v>60</v>
       </c>
       <c r="O46" s="7" t="n">
-        <v>45963.3376273148</v>
+        <v>45700.7520138889</v>
       </c>
       <c r="P46" s="6"/>
       <c r="Q46" s="7"/>
-      <c r="R46" s="6"/>
+      <c r="R46" s="6" t="s">
+        <v>162</v>
+      </c>
       <c r="S46" s="6" t="s">
         <v>28</v>
       </c>
@@ -3525,13 +3536,13 @@
     </row>
     <row r="47" customHeight="1" ht="20">
       <c r="A47" s="5" t="n">
-        <v>781</v>
+        <v>761</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D47" s="5" t="n">
         <v>6</v>
@@ -3543,7 +3554,7 @@
         <v>24</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>880</v>
+        <v>1000</v>
       </c>
       <c r="H47" s="6" t="s">
         <v>56</v>
@@ -3565,7 +3576,7 @@
         <v>60</v>
       </c>
       <c r="O47" s="7" t="n">
-        <v>45964.9283101852</v>
+        <v>45963.3376273148</v>
       </c>
       <c r="P47" s="6"/>
       <c r="Q47" s="7"/>
@@ -3578,27 +3589,27 @@
       <c r="V47" s="6"/>
       <c r="W47" s="6"/>
     </row>
-    <row r="48" customHeight="1" ht="29">
+    <row r="48" customHeight="1" ht="20">
       <c r="A48" s="5" t="n">
-        <v>42</v>
+        <v>781</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D48" s="5" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>2300</v>
+        <v>880</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>56</v>
@@ -3608,25 +3619,23 @@
         <v>1</v>
       </c>
       <c r="K48" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="L48" s="5" t="n">
-        <v>148</v>
+        <v>110</v>
       </c>
       <c r="M48" s="5" t="n">
         <v>10</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="O48" s="7" t="n">
-        <v>44445.445150463</v>
+        <v>45964.9283101852</v>
       </c>
       <c r="P48" s="6"/>
       <c r="Q48" s="7"/>
-      <c r="R48" s="6" t="s">
-        <v>166</v>
-      </c>
+      <c r="R48" s="6"/>
       <c r="S48" s="6" t="s">
         <v>28</v>
       </c>
@@ -3635,9 +3644,9 @@
       <c r="V48" s="6"/>
       <c r="W48" s="6"/>
     </row>
-    <row r="49" customHeight="1" ht="43,5">
+    <row r="49" customHeight="1" ht="29">
       <c r="A49" s="5" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B49" s="6" t="s">
         <v>167</v>
@@ -3646,19 +3655,19 @@
         <v>168</v>
       </c>
       <c r="D49" s="5" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="F49" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>600</v>
+        <v>2300</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="I49" s="6"/>
       <c r="J49" s="5" t="n">
@@ -3668,7 +3677,7 @@
         <v>13</v>
       </c>
       <c r="L49" s="5" t="n">
-        <v>110</v>
+        <v>148</v>
       </c>
       <c r="M49" s="5" t="n">
         <v>10</v>
@@ -3677,7 +3686,7 @@
         <v>26</v>
       </c>
       <c r="O49" s="7" t="n">
-        <v>44445.4470717593</v>
+        <v>44445.445150463</v>
       </c>
       <c r="P49" s="6"/>
       <c r="Q49" s="7"/>
@@ -3692,9 +3701,9 @@
       <c r="V49" s="6"/>
       <c r="W49" s="6"/>
     </row>
-    <row r="50" customHeight="1" ht="29">
+    <row r="50" customHeight="1" ht="43,5">
       <c r="A50" s="5" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B50" s="6" t="s">
         <v>170</v>
@@ -3734,14 +3743,10 @@
         <v>26</v>
       </c>
       <c r="O50" s="7" t="n">
-        <v>44445</v>
-      </c>
-      <c r="P50" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q50" s="7" t="n">
-        <v>45479.6319907407</v>
-      </c>
+        <v>44445.4470717593</v>
+      </c>
+      <c r="P50" s="6"/>
+      <c r="Q50" s="7"/>
       <c r="R50" s="6" t="s">
         <v>172</v>
       </c>
@@ -3753,9 +3758,9 @@
       <c r="V50" s="6"/>
       <c r="W50" s="6"/>
     </row>
-    <row r="51" customHeight="1" ht="72,5">
+    <row r="51" customHeight="1" ht="29">
       <c r="A51" s="5" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B51" s="6" t="s">
         <v>173</v>
@@ -3764,16 +3769,16 @@
         <v>174</v>
       </c>
       <c r="D51" s="5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F51" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>280</v>
+        <v>600</v>
       </c>
       <c r="H51" s="6" t="s">
         <v>25</v>
@@ -3795,10 +3800,14 @@
         <v>26</v>
       </c>
       <c r="O51" s="7" t="n">
-        <v>44445.4529976852</v>
-      </c>
-      <c r="P51" s="6"/>
-      <c r="Q51" s="7"/>
+        <v>44445</v>
+      </c>
+      <c r="P51" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q51" s="7" t="n">
+        <v>45479.6319907407</v>
+      </c>
       <c r="R51" s="6" t="s">
         <v>175</v>
       </c>
@@ -3810,9 +3819,9 @@
       <c r="V51" s="6"/>
       <c r="W51" s="6"/>
     </row>
-    <row r="52" customHeight="1" ht="43,5">
+    <row r="52" customHeight="1" ht="72,5">
       <c r="A52" s="5" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B52" s="6" t="s">
         <v>176</v>
@@ -3821,16 +3830,16 @@
         <v>177</v>
       </c>
       <c r="D52" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>140</v>
+        <v>280</v>
       </c>
       <c r="H52" s="6" t="s">
         <v>25</v>
@@ -3840,19 +3849,19 @@
         <v>1</v>
       </c>
       <c r="K52" s="5" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="L52" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M52" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O52" s="7" t="n">
-        <v>44445.4599768519</v>
+        <v>44445.4529976852</v>
       </c>
       <c r="P52" s="6"/>
       <c r="Q52" s="7"/>
@@ -3862,36 +3871,32 @@
       <c r="S52" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="T52" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="U52" s="6" t="s">
-        <v>179</v>
-      </c>
+      <c r="T52" s="6"/>
+      <c r="U52" s="6"/>
       <c r="V52" s="6"/>
       <c r="W52" s="6"/>
     </row>
-    <row r="53" customHeight="1" ht="101,5">
+    <row r="53" customHeight="1" ht="43,5">
       <c r="A53" s="5" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C53" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C53" s="6" t="s">
-        <v>181</v>
-      </c>
       <c r="D53" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="H53" s="6" t="s">
         <v>25</v>
@@ -3901,36 +3906,40 @@
         <v>1</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L53" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M53" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N53" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O53" s="7" t="n">
-        <v>44445.4633449074</v>
+        <v>44445.4599768519</v>
       </c>
       <c r="P53" s="6"/>
       <c r="Q53" s="7"/>
       <c r="R53" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="S53" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T53" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="U53" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="S53" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T53" s="6"/>
-      <c r="U53" s="6"/>
       <c r="V53" s="6"/>
       <c r="W53" s="6"/>
     </row>
-    <row r="54" customHeight="1" ht="72,5">
+    <row r="54" customHeight="1" ht="101,5">
       <c r="A54" s="5" t="n">
-        <v>141</v>
+        <v>54</v>
       </c>
       <c r="B54" s="6" t="s">
         <v>183</v>
@@ -3939,38 +3948,38 @@
         <v>184</v>
       </c>
       <c r="D54" s="5" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G54" s="5" t="n">
-        <v>2000</v>
+        <v>230</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I54" s="6"/>
       <c r="J54" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L54" s="5" t="n">
-        <v>226</v>
+        <v>110</v>
       </c>
       <c r="M54" s="5" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="N54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O54" s="7" t="n">
-        <v>44791.3073842593</v>
+        <v>44445.4633449074</v>
       </c>
       <c r="P54" s="6"/>
       <c r="Q54" s="7"/>
@@ -3985,53 +3994,55 @@
       <c r="V54" s="6"/>
       <c r="W54" s="6"/>
     </row>
-    <row r="55" customHeight="1" ht="20">
+    <row r="55" customHeight="1" ht="72,5">
       <c r="A55" s="5" t="n">
-        <v>381</v>
+        <v>141</v>
       </c>
       <c r="B55" s="6" t="s">
         <v>186</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D55" s="5" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>250</v>
+        <v>2000</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="I55" s="6"/>
       <c r="J55" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K55" s="5" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="L55" s="5" t="n">
-        <v>110</v>
+        <v>226</v>
       </c>
       <c r="M55" s="5" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="N55" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O55" s="7" t="n">
-        <v>45082.6267476852</v>
+        <v>44791.3073842593</v>
       </c>
       <c r="P55" s="6"/>
       <c r="Q55" s="7"/>
-      <c r="R55" s="6"/>
+      <c r="R55" s="6" t="s">
+        <v>188</v>
+      </c>
       <c r="S55" s="6" t="s">
         <v>28</v>
       </c>
@@ -4042,35 +4053,35 @@
     </row>
     <row r="56" customHeight="1" ht="20">
       <c r="A56" s="5" t="n">
-        <v>561</v>
+        <v>381</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D56" s="5" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I56" s="6"/>
       <c r="J56" s="5" t="n">
         <v>1</v>
       </c>
       <c r="K56" s="5" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L56" s="5" t="n">
         <v>110</v>
@@ -4082,13 +4093,11 @@
         <v>26</v>
       </c>
       <c r="O56" s="7" t="n">
-        <v>45646.6471527778</v>
+        <v>45082.6267476852</v>
       </c>
       <c r="P56" s="6"/>
       <c r="Q56" s="7"/>
-      <c r="R56" s="6" t="s">
-        <v>189</v>
-      </c>
+      <c r="R56" s="6"/>
       <c r="S56" s="6" t="s">
         <v>28</v>
       </c>
@@ -4099,7 +4108,7 @@
     </row>
     <row r="57" customHeight="1" ht="20">
       <c r="A57" s="5" t="n">
-        <v>801</v>
+        <v>561</v>
       </c>
       <c r="B57" s="6" t="s">
         <v>190</v>
@@ -4108,16 +4117,16 @@
         <v>191</v>
       </c>
       <c r="D57" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E57" s="5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="H57" s="6" t="s">
         <v>56</v>
@@ -4127,7 +4136,7 @@
         <v>1</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="L57" s="5" t="n">
         <v>110</v>
@@ -4136,14 +4145,16 @@
         <v>10</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="O57" s="7" t="n">
-        <v>45981.747025463</v>
+        <v>45646.6471527778</v>
       </c>
       <c r="P57" s="6"/>
       <c r="Q57" s="7"/>
-      <c r="R57" s="6"/>
+      <c r="R57" s="6" t="s">
+        <v>192</v>
+      </c>
       <c r="S57" s="6" t="s">
         <v>28</v>
       </c>
@@ -4154,32 +4165,32 @@
     </row>
     <row r="58" customHeight="1" ht="20">
       <c r="A58" s="5" t="n">
-        <v>822</v>
+        <v>801</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D58" s="5" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E58" s="5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>700</v>
+        <v>1200</v>
       </c>
       <c r="H58" s="6" t="s">
         <v>56</v>
       </c>
       <c r="I58" s="6"/>
       <c r="J58" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K58" s="5" t="n">
         <v>14</v>
@@ -4194,7 +4205,7 @@
         <v>60</v>
       </c>
       <c r="O58" s="7" t="n">
-        <v>45983.3518402778</v>
+        <v>45981.747025463</v>
       </c>
       <c r="P58" s="6"/>
       <c r="Q58" s="7"/>
@@ -4207,55 +4218,53 @@
       <c r="V58" s="6"/>
       <c r="W58" s="6"/>
     </row>
-    <row r="59" customHeight="1" ht="58">
+    <row r="59" customHeight="1" ht="20">
       <c r="A59" s="5" t="n">
-        <v>161</v>
+        <v>822</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D59" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G59" s="5" t="n">
-        <v>120</v>
+        <v>700</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
       <c r="I59" s="6"/>
       <c r="J59" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="L59" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M59" s="5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="O59" s="7" t="n">
-        <v>44807.6812268519</v>
+        <v>45983.3518402778</v>
       </c>
       <c r="P59" s="6"/>
       <c r="Q59" s="7"/>
-      <c r="R59" s="6" t="s">
-        <v>196</v>
-      </c>
+      <c r="R59" s="6"/>
       <c r="S59" s="6" t="s">
         <v>28</v>
       </c>
@@ -4264,9 +4273,9 @@
       <c r="V59" s="6"/>
       <c r="W59" s="6"/>
     </row>
-    <row r="60" customHeight="1" ht="20">
+    <row r="60" customHeight="1" ht="58">
       <c r="A60" s="5" t="n">
-        <v>361</v>
+        <v>161</v>
       </c>
       <c r="B60" s="6" t="s">
         <v>197</v>
@@ -4275,16 +4284,16 @@
         <v>198</v>
       </c>
       <c r="D60" s="5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E60" s="5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>550</v>
+        <v>120</v>
       </c>
       <c r="H60" s="6" t="s">
         <v>25</v>
@@ -4294,27 +4303,25 @@
         <v>1</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="L60" s="5" t="n">
         <v>110</v>
       </c>
       <c r="M60" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N60" s="6" t="s">
         <v>26</v>
       </c>
       <c r="O60" s="7" t="n">
-        <v>45069</v>
-      </c>
-      <c r="P60" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q60" s="7" t="n">
-        <v>45069.5181018519</v>
-      </c>
-      <c r="R60" s="6"/>
+        <v>44807.6812268519</v>
+      </c>
+      <c r="P60" s="6"/>
+      <c r="Q60" s="7"/>
+      <c r="R60" s="6" t="s">
+        <v>199</v>
+      </c>
       <c r="S60" s="6" t="s">
         <v>28</v>
       </c>
@@ -4325,35 +4332,35 @@
     </row>
     <row r="61" customHeight="1" ht="20">
       <c r="A61" s="5" t="n">
-        <v>681</v>
+        <v>361</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D61" s="5" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>1200</v>
+        <v>550</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="I61" s="6"/>
       <c r="J61" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L61" s="5" t="n">
         <v>110</v>
@@ -4362,16 +4369,18 @@
         <v>10</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="O61" s="7" t="n">
-        <v>45793.6175462963</v>
-      </c>
-      <c r="P61" s="6"/>
-      <c r="Q61" s="7"/>
-      <c r="R61" s="6" t="s">
-        <v>201</v>
-      </c>
+        <v>45069</v>
+      </c>
+      <c r="P61" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q61" s="7" t="n">
+        <v>45069.5181018519</v>
+      </c>
+      <c r="R61" s="6"/>
       <c r="S61" s="6" t="s">
         <v>28</v>
       </c>
@@ -4382,7 +4391,7 @@
     </row>
     <row r="62" customHeight="1" ht="20">
       <c r="A62" s="5" t="n">
-        <v>623</v>
+        <v>681</v>
       </c>
       <c r="B62" s="6" t="s">
         <v>202</v>
@@ -4397,17 +4406,17 @@
         <v>6</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>1000</v>
+        <v>1200</v>
       </c>
       <c r="H62" s="6" t="s">
         <v>56</v>
       </c>
       <c r="I62" s="6"/>
       <c r="J62" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K62" s="5" t="n">
         <v>14</v>
@@ -4422,7 +4431,7 @@
         <v>60</v>
       </c>
       <c r="O62" s="7" t="n">
-        <v>45700.7507407407</v>
+        <v>45793.6175462963</v>
       </c>
       <c r="P62" s="6"/>
       <c r="Q62" s="7"/>
@@ -4439,7 +4448,7 @@
     </row>
     <row r="63" customHeight="1" ht="20">
       <c r="A63" s="5" t="n">
-        <v>722</v>
+        <v>623</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>205</v>
@@ -4448,16 +4457,16 @@
         <v>206</v>
       </c>
       <c r="D63" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>56</v>
@@ -4479,11 +4488,13 @@
         <v>60</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>45908.4576388889</v>
+        <v>45700.7507407407</v>
       </c>
       <c r="P63" s="6"/>
       <c r="Q63" s="7"/>
-      <c r="R63" s="6"/>
+      <c r="R63" s="6" t="s">
+        <v>207</v>
+      </c>
       <c r="S63" s="6" t="s">
         <v>28</v>
       </c>
@@ -4491,6 +4502,61 @@
       <c r="U63" s="6"/>
       <c r="V63" s="6"/>
       <c r="W63" s="6"/>
+    </row>
+    <row r="64" customHeight="1" ht="20">
+      <c r="A64" s="5" t="n">
+        <v>722</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D64" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E64" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G64" s="5" t="n">
+        <v>1100</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I64" s="6"/>
+      <c r="J64" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="L64" s="5" t="n">
+        <v>110</v>
+      </c>
+      <c r="M64" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="N64" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="O64" s="7" t="n">
+        <v>45908.4576388889</v>
+      </c>
+      <c r="P64" s="6"/>
+      <c r="Q64" s="7"/>
+      <c r="R64" s="6"/>
+      <c r="S64" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T64" s="6"/>
+      <c r="U64" s="6"/>
+      <c r="V64" s="6"/>
+      <c r="W64" s="6"/>
     </row>
   </sheetData>
   <tableParts count="1">

</xml_diff>

<commit_message>
Feat: Complete logic for Participant Management with Intolerance Icons and optimized Header loading
</commit_message>
<xml_diff>
--- a/inp_Excel/ana_viaggi.xlsx
+++ b/inp_Excel/ana_viaggi.xlsx
@@ -9,7 +9,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="207">
   <si>
     <t>VIAGGIO_ID</t>
   </si>
@@ -655,15 +655,6 @@
   </si>
   <si>
     <t>https://www.sardegnafuoritraccia.it/it/tour/moto-enduro/maxi-enduro-tour-gpx-sardegna-2025</t>
-  </si>
-  <si>
-    <t>ICHNUSA TOUR 4X4</t>
-  </si>
-  <si>
-    <t>GIRO DELLA SARDEGNA IN FUORISTRADA</t>
-  </si>
-  <si>
-    <t>https://www.sardegnafuoritraccia.it/it/tour/fuoristrada/ichnusa-tour-4x4</t>
   </si>
   <si>
     <t>CAPODANNO IN FUORISTRADA 8 GG</t>
@@ -769,8 +760,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:W64" totalsRowShown="0" headerRowCount="1">
-  <autoFilter ref="A1:W64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" displayName="foglio1" ref="A1:W63" totalsRowShown="0" headerRowCount="1">
+  <autoFilter ref="A1:W63"/>
   <tableColumns count="23">
     <tableColumn id="1" name="VIAGGIO_ID"/>
     <tableColumn id="2" name="VIAGGIO_DESCRIZIONE_BREVE"/>
@@ -4448,7 +4439,7 @@
     </row>
     <row r="63" customHeight="1" ht="20">
       <c r="A63" s="5" t="n">
-        <v>623</v>
+        <v>722</v>
       </c>
       <c r="B63" s="6" t="s">
         <v>205</v>
@@ -4457,16 +4448,16 @@
         <v>206</v>
       </c>
       <c r="D63" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E63" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="E63" s="5" t="n">
-        <v>6</v>
-      </c>
       <c r="F63" s="6" t="s">
         <v>24</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="H63" s="6" t="s">
         <v>56</v>
@@ -4488,13 +4479,11 @@
         <v>60</v>
       </c>
       <c r="O63" s="7" t="n">
-        <v>45700.7507407407</v>
+        <v>45908.4576388889</v>
       </c>
       <c r="P63" s="6"/>
       <c r="Q63" s="7"/>
-      <c r="R63" s="6" t="s">
-        <v>207</v>
-      </c>
+      <c r="R63" s="6"/>
       <c r="S63" s="6" t="s">
         <v>28</v>
       </c>
@@ -4502,61 +4491,6 @@
       <c r="U63" s="6"/>
       <c r="V63" s="6"/>
       <c r="W63" s="6"/>
-    </row>
-    <row r="64" customHeight="1" ht="20">
-      <c r="A64" s="5" t="n">
-        <v>722</v>
-      </c>
-      <c r="B64" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D64" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E64" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="G64" s="5" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I64" s="6"/>
-      <c r="J64" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K64" s="5" t="n">
-        <v>14</v>
-      </c>
-      <c r="L64" s="5" t="n">
-        <v>110</v>
-      </c>
-      <c r="M64" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="O64" s="7" t="n">
-        <v>45908.4576388889</v>
-      </c>
-      <c r="P64" s="6"/>
-      <c r="Q64" s="7"/>
-      <c r="R64" s="6"/>
-      <c r="S64" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="T64" s="6"/>
-      <c r="U64" s="6"/>
-      <c r="V64" s="6"/>
-      <c r="W64" s="6"/>
     </row>
   </sheetData>
   <tableParts count="1">

</xml_diff>